<commit_message>
Outline draft and test result reorganise
</commit_message>
<xml_diff>
--- a/Testing Data/Alter-layer Specimen Testing.xlsx
+++ b/Testing Data/Alter-layer Specimen Testing.xlsx
@@ -684,10 +684,18 @@
       <c r="H5" s="17"/>
       <c r="I5" s="16"/>
       <c r="J5" s="17"/>
-      <c r="K5" s="16"/>
-      <c r="L5" s="17"/>
-      <c r="M5" s="16"/>
-      <c r="N5" s="18"/>
+      <c r="K5" s="16" t="n">
+        <v>139</v>
+      </c>
+      <c r="L5" s="17" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="M5" s="16" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="N5" s="18" t="n">
+        <v>125</v>
+      </c>
       <c r="O5" s="1" t="s">
         <v>7</v>
       </c>
@@ -750,10 +758,18 @@
       <c r="H7" s="17"/>
       <c r="I7" s="16"/>
       <c r="J7" s="17"/>
-      <c r="K7" s="16"/>
-      <c r="L7" s="17"/>
-      <c r="M7" s="16"/>
-      <c r="N7" s="18"/>
+      <c r="K7" s="16" t="n">
+        <v>116</v>
+      </c>
+      <c r="L7" s="17" t="n">
+        <v>108</v>
+      </c>
+      <c r="M7" s="16" t="n">
+        <v>117</v>
+      </c>
+      <c r="N7" s="18" t="n">
+        <v>125</v>
+      </c>
       <c r="O7" s="1" t="s">
         <v>8</v>
       </c>
@@ -814,10 +830,18 @@
       <c r="H9" s="17"/>
       <c r="I9" s="16"/>
       <c r="J9" s="17"/>
-      <c r="K9" s="16"/>
-      <c r="L9" s="17"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="18"/>
+      <c r="K9" s="16" t="n">
+        <v>109</v>
+      </c>
+      <c r="L9" s="17" t="n">
+        <v>104</v>
+      </c>
+      <c r="M9" s="16" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="N9" s="18" t="n">
+        <v>107.5</v>
+      </c>
       <c r="O9" s="1" t="s">
         <v>9</v>
       </c>

</xml_diff>